<commit_message>
v1.3.3: 修复 7 个 bug + _active.xlsx 去副本化 + Claude Code 行为约束
Bug 修复:
- B4: loadIssues 重复 catch 死代码导致 JS SyntaxError，前端不可用
- B5: detect_columns 后面列覆盖前面列映射
- B6: result_col 误匹配 Pass/Fail 列
- B7: read_testcases 改用 SAVE_COLUMNS 精确列名匹配
- B8: 自动识别 testcases 中任意 Excel 作为活跃文件
- B9: _pick_best_sheet 优先选有测试结果列的 Sheet
- B10: 移除 _active.xlsx 副本，直接读写原始 Excel (方案 A)

新功能:
- 测试人员/BugID/Bug频率(必现/高频/偶现/1次)/问题时间(失败自动记录)
- 问题列表第4标签页 + 全通过庆祝动画
- 搜索结果显示用例名称
- 前置条件蓝色边框、操作区 2x2 网格 UI 美化

文档:
- CLAUDE.md 新增 Claude Code 行为约束（防死循环/防重复打开浏览器）
</commit_message>
<xml_diff>
--- a/testcases/货架偏移容差测试用例.xlsx
+++ b/testcases/货架偏移容差测试用例.xlsx
@@ -8005,7 +8005,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="16.5" customHeight="1">
       <c r="A3" s="17" t="inlineStr">
         <is>
@@ -8594,7 +8593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J66"/>
+  <dimension ref="A1:P66"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8672,6 +8671,36 @@
           <t>备注</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>实际结果</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>测试人员</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>BugID</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Bug频率</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>问题时间</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>执行时间</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -8704,10 +8733,29 @@
           <t>基准</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr"/>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
       <c r="H4" s="9" t="inlineStr"/>
       <c r="I4" s="9" t="inlineStr"/>
       <c r="J4" s="9" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>直接写入原始文件ok</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>张三</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>2026-07-05 10:23:57</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -10808,7 +10856,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="16.5" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: 阶段4 清理补测 - 补 API 测试 + ESLint 配置 + Makefile 修复
新增内容：
1. 补 8 个 API 路由测试（tests/test_testcase_viewer.py）：
   - TestApiTitles: /api/titles 已加载/未加载
   - TestApiReload: /api/reload 成功/无文件
   - TestApiUpload: /api/upload 无文件/空文件名/错误格式
   - TestApiCheckResults: /api/check-results 响应格式
   覆盖率 64% → 70%

2. 前端 ESLint 配置：
   - package.json（声明 eslint 依赖，未来 npm install 启用）
   - .eslintrc.json（规则：no-undef/no-dupe-keys/no-unreachable 等）
   - 当前环境网络不通无法装 eslint，用 node --check 替代（能抓 B4 那种语法错误）

3. Makefile 修复：
   - python → $(PYTHON) 默认 /usr/bin/python3（有 pytest 的环境）
   - pip → pip3
   - lint 命令拆 lint-py + lint-js，工具未装时优雅降级（py_compile 替代）
   - 新增 lint-js 目标（node --check，零依赖）
   - format 命令工具未装时提示安装方法

验证：43 passed 全绿；make lint 通过（Python 语法 + JS 语法）
</commit_message>
<xml_diff>
--- a/testcases/货架偏移容差测试用例.xlsx
+++ b/testcases/货架偏移容差测试用例.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowHeight="19240" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="货架偏移容差测试用例" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="偏移场景说明" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统计汇总" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试记录表(填写用)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="判定标准与执行说明" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="货架偏移容差测试用例" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="偏移场景说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="统计汇总" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="测试记录表(填写用)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="判定标准与执行说明" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'货架偏移容差测试用例'!$A$3:$U$66</definedName>
@@ -1568,7 +1568,7 @@
       <c r="Z4" s="20" t="inlineStr"/>
       <c r="AA4" s="20" t="inlineStr">
         <is>
-          <t>2026-07-07 23:06:01</t>
+          <t>2026-07-08 00:24:20</t>
         </is>
       </c>
     </row>

</xml_diff>